<commit_message>
Any class can be coach or coachee; Teams intro links per pair
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Martinson_Matching_SAMPLE.xlsx
+++ b/Martinson_Matching_SAMPLE.xlsx
@@ -129,8 +129,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Responses" displayName="Responses" ref="A1:P25" headerRowCount="1">
-  <autoFilter ref="A1:P25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Responses" displayName="Responses" ref="A1:P29" headerRowCount="1">
+  <autoFilter ref="A1:P29"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Name"/>
     <tableColumn id="2" name="Email"/>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -553,12 +553,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>C29Alex.Nguyen@example.com</t>
+          <t>C28Alex.Nguyen@example.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2029</t>
+          <t>2028</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -626,17 +626,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jordan Patel</t>
+          <t>Jordan Johnson</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>C29Jordan.Patel@example.com</t>
+          <t>C28Jordan.Johnson@example.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2029</t>
+          <t>2028</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -704,17 +704,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sam Lopez</t>
+          <t>Sam Wilson</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>C29Sam.Lopez@example.com</t>
+          <t>C28Sam.Wilson@example.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2029</t>
+          <t>2028</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -782,17 +782,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Riley Martinez</t>
+          <t>Riley Smith</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>C29Riley.Martinez@example.com</t>
+          <t>C28Riley.Smith@example.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2029</t>
+          <t>2028</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -860,12 +860,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Taylor Thomas</t>
+          <t>Taylor Lopez</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C29Taylor.Thomas@example.com</t>
+          <t>C29Taylor.Lopez@example.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -938,12 +938,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Morgan Smith</t>
+          <t>Morgan Anderson</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C29Morgan.Smith@example.com</t>
+          <t>C29Morgan.Anderson@example.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1016,12 +1016,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Casey Kim</t>
+          <t>Casey Garcia</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>C29Casey.Kim@example.com</t>
+          <t>C29Casey.Garcia@example.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1172,12 +1172,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Avery Wilson</t>
+          <t>Avery Thomas</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>C29Avery.Wilson@example.com</t>
+          <t>C29Avery.Thomas@example.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1250,12 +1250,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Quinn Moore</t>
+          <t>Quinn Patel</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>C29Quinn.Moore@example.com</t>
+          <t>C29Quinn.Patel@example.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1328,17 +1328,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Drew Garcia</t>
+          <t>Drew Davis</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>C30Drew.Garcia@example.com</t>
+          <t>C29Drew.Davis@example.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2030</t>
+          <t>2029</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1406,17 +1406,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Reese Johnson</t>
+          <t>Reese Moore</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>C30Reese.Johnson@example.com</t>
+          <t>C29Reese.Moore@example.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2030</t>
+          <t>2029</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1484,17 +1484,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Skyler Davis</t>
+          <t>Skyler Kim</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>C30Skyler.Davis@example.com</t>
+          <t>C29Skyler.Kim@example.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2030</t>
+          <t>2029</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1562,17 +1562,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Parker Anderson</t>
+          <t>Parker Martinez</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>C30Parker.Anderson@example.com</t>
+          <t>C29Parker.Martinez@example.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2030</t>
+          <t>2029</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1718,12 +1718,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Emerson Patel</t>
+          <t>Emerson Johnson</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>C30Emerson.Patel@example.com</t>
+          <t>C30Emerson.Johnson@example.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1796,12 +1796,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Hayden Lopez</t>
+          <t>Hayden Wilson</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>C30Hayden.Lopez@example.com</t>
+          <t>C30Hayden.Wilson@example.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1874,12 +1874,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Kendall Martinez</t>
+          <t>Kendall Smith</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>C30Kendall.Martinez@example.com</t>
+          <t>C30Kendall.Smith@example.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1952,12 +1952,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Logan Thomas</t>
+          <t>Logan Lopez</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>C30Logan.Thomas@example.com</t>
+          <t>C30Logan.Lopez@example.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2030,12 +2030,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Blake Smith</t>
+          <t>Blake Anderson</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>C30Blake.Smith@example.com</t>
+          <t>C30Blake.Anderson@example.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2108,12 +2108,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Cameron Kim</t>
+          <t>Cameron Garcia</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>C30Cameron.Kim@example.com</t>
+          <t>C30Cameron.Garcia@example.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2264,12 +2264,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Elliot Wilson</t>
+          <t>Elliot Thomas</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>C30Elliot.Wilson@example.com</t>
+          <t>C30Elliot.Thomas@example.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2342,12 +2342,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Finley Moore</t>
+          <t>Finley Patel</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>C30Finley.Moore@example.com</t>
+          <t>C30Finley.Patel@example.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2416,6 +2416,318 @@
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Alex Martinez</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>C30Alex.Martinez@example.com</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2030</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Academics &amp; study habits;</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Economics;Meteorology;Chemistry;</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Nuclear Weapons &amp; Strategy;</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Master's right after graduation;Gates Cambridge;</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Missiles;</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Career military;Law;</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Cadet leadership positions;Publishing research;Ops Air Force;</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Aerospace / hypersonics;AI / machine learning;History;</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>I'm interested in quantum sensing and cyber defense of space systems.</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Skiing / snowboarding;Writing;Gaming;</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Mentorship / first-gen students;</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Jordan Nguyen</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>C30Jordan.Nguyen@example.com</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2030</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>["Leadership &amp; military training"]</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>["Electrical &amp; Computer Engineering", "Economics"]</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>["Nuclear Weapons &amp; Strategy", "Global Logistics"]</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>["Medical school", "Schwarzman", "Mitchell"]</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>["Developmental Engineer", "Acquisitions / Program Management", "Medical"]</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>["Law", "Career military", "Industry / tech"]</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>["Study abroad / exchange semester", "Internships", "Ops Air Force"]</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>["Education", "Quantum / physics", "Space"]</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>I'm interested in cyber defense of space systems and human performance and sleep.</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>["Volunteering", "Skiing / snowboarding"]</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>["Climate", "Economic opportunity", "Education access"]</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Sam Johnson</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>C30Sam.Johnson@example.com</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2030</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Time management;Choosing a major;</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Cyber Science;English;</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Space Studies;Foreign language;</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Not planning grad school;Mitchell;Not sure yet;</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>JAG;Intelligence;</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Entrepreneurship;Academia / research;</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Competition teams / clubs;</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>History;Aerospace / hypersonics;</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>I'm interested in renewable energy on bases and great power competition.</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Music;Climbing;Skiing / snowboarding;</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Community service;</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Riley Wilson</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>C30Riley.Wilson@example.com</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2030</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>["Leadership &amp; military training", "Navigating cadet life", "AF/SF career planning"]</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>["Chemistry"]</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>["Other"]</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>["Not sure yet", "Not planning grad school", "Hertz / NSF GRFP"]</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>["Medical", "Pilot", "RPA Pilot"]</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>["Not sure yet", "Government / policy"]</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>["Internships"]</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>["Cybersecurity"]</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>I'm interested in machine learning for satellite imagery and great power competition.</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>["Hiking / outdoors", "Travel", "Lifting"]</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>["Mental health", "Economic opportunity", "Veterans"]</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Drop Issues question; reword coaching focus
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Martinson_Matching_SAMPLE.xlsx
+++ b/Martinson_Matching_SAMPLE.xlsx
@@ -129,9 +129,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Responses" displayName="Responses" ref="A1:P29" headerRowCount="1">
-  <autoFilter ref="A1:P29"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Responses" displayName="Responses" ref="A1:O29" headerRowCount="1">
+  <autoFilter ref="A1:O29"/>
+  <tableColumns count="15">
     <tableColumn id="1" name="Name"/>
     <tableColumn id="2" name="Email"/>
     <tableColumn id="3" name="Class Year"/>
@@ -146,8 +146,7 @@
     <tableColumn id="12" name="Research Areas"/>
     <tableColumn id="13" name="Research Interests"/>
     <tableColumn id="14" name="Fun"/>
-    <tableColumn id="15" name="Issues"/>
-    <tableColumn id="16" name="Anything Else"/>
+    <tableColumn id="15" name="Anything Else"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -442,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -460,7 +459,6 @@
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -536,11 +534,6 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Issues</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
           <t>Anything Else</t>
         </is>
       </c>
@@ -616,12 +609,7 @@
           <t>Gaming;</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Economic opportunity;Faith &amp; values;Mental health;</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -641,65 +629,60 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>["Navigating cadet life", "Academics &amp; study habits", "Grad school planning"]</t>
+          <t>["Wellness &amp; balance"]</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>["Management"]</t>
+          <t>["Foreign Area Studies", "Astronautical Engineering", "Cyber Science"]</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>["Nuclear Weapons &amp; Strategy"]</t>
+          <t>["Religion Studies"]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>["Fulbright", "Master's right after graduation"]</t>
+          <t>["Mitchell", "Fulbright"]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>["Finance / Contracting"]</t>
+          <t>["Air Battle Manager", "Finance / Contracting", "Acquisitions / Program Management"]</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>["Academia / research", "Career military"]</t>
+          <t>["Academia / research", "Career military", "Entrepreneurship"]</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>["Conferences / presenting", "Ops Air Force", "Jump"]</t>
+          <t>["Ops Air Force", "Jump", "Internships"]</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>["Aerospace / hypersonics"]</t>
+          <t>["Aerospace / hypersonics", "Materials", "AI / machine learning"]</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>I'm interested in leadership psychology under stress and swarm autonomy for drones.</t>
+          <t>I'm interested in leadership psychology under stress and ethics of autonomous weapons.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>["Music", "Film / TV", "Art / photography"]</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>["Community service", "Global security", "Healthcare"]</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr"/>
+          <t>["Volunteering", "Art / photography"]</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -719,12 +702,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Research opportunities;AF/SF career planning;</t>
+          <t>Leadership &amp; military training;Research opportunities;AF/SF career planning;</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -772,12 +755,7 @@
           <t>Lifting;Climbing;</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Faith &amp; values;Global security;Economic opportunity;</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -797,65 +775,60 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>36</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>["Leadership &amp; military training", "Wellness &amp; balance", "Choosing a major"]</t>
+          <t>["Research opportunities", "Wellness &amp; balance", "Time management"]</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>["Data Science"]</t>
+          <t>["Humanities", "Mathematics", "Political Science"]</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["Philosophy", "Foreign language"]</t>
+          <t>["Philosophy", "Other"]</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>["Law school", "Schwarzman", "Medical school"]</t>
+          <t>["Schwarzman"]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>["OSI", "Acquisitions / Program Management", "Maintenance / Logistics"]</t>
+          <t>["RPA Pilot", "Combat Systems Officer"]</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>["Medicine", "Career military", "Government / policy"]</t>
+          <t>["Entrepreneurship", "Medicine", "Not sure yet"]</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>["Study abroad / exchange semester", "Internships"]</t>
+          <t>["Competition teams / clubs", "Soaring / powered flight", "Cadet leadership positions"]</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>["Autonomy / drones", "Space"]</t>
+          <t>["History", "AI / machine learning", "Climate / environment"]</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>I'm interested in Cold War nuclear strategy and machine learning for satellite imagery.</t>
+          <t>I'm interested in human performance and sleep and machine learning for satellite imagery.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>["Gaming", "Faith community", "Music"]</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>["Education access", "Veterans"]</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr"/>
+          <t>["Hiking / outdoors", "Film / TV", "Running"]</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -875,65 +848,60 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Time management;AF/SF career planning;</t>
+          <t>Fellowships &amp; scholarships;Grad school planning;</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Space Operations;</t>
+          <t>Foreign Area Studies;Systems Engineering;</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Nuclear Weapons &amp; Strategy;Global Logistics;</t>
+          <t>Philosophy;None / undecided;</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Gates Cambridge;Medical school;</t>
+          <t>Mitchell;Master's right after graduation;</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Developmental Engineer;Space Operations;</t>
+          <t>Space Operations;Security Forces;</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Academia / research;</t>
+          <t>Entrepreneurship;Medicine;Government / policy;</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Ops Air Force;</t>
+          <t>Cadet leadership positions;Ops Air Force;</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Climate / environment;AI / machine learning;Education;</t>
+          <t>Aerospace / hypersonics;</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>I'm interested in leadership psychology under stress and machine learning for satellite imagery.</t>
+          <t>I'm interested in machine learning for satellite imagery and machine learning for satellite imagery.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Writing;Running;</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Community service;</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr"/>
+          <t>Gaming;</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -953,65 +921,60 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>["Wellness &amp; balance", "Research opportunities"]</t>
+          <t>["Wellness &amp; balance", "Fellowships &amp; scholarships"]</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>["Operations Research"]</t>
+          <t>["Economics", "Aeronautical Engineering"]</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["Foreign language", "Space Studies", "Global Logistics"]</t>
+          <t>["Other"]</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>["Mitchell", "Not planning grad school", "Not sure yet"]</t>
+          <t>["Gates Cambridge", "PhD", "Not sure yet"]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>["Air Battle Manager", "Medical"]</t>
+          <t>["Space Operations", "JAG"]</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>["Law", "Career military", "Industry / tech"]</t>
+          <t>["Career military", "Government / policy", "Medicine"]</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>["Ops Air Force"]</t>
+          <t>["Cadet leadership positions", "Conferences / presenting", "Publishing research"]</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>["Energy", "Autonomy / drones"]</t>
+          <t>["Space", "Climate / environment"]</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>I'm interested in human performance and sleep and leadership psychology under stress.</t>
+          <t>I'm interested in renewable energy on bases and quantum sensing.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>["Hiking / outdoors"]</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>["Faith &amp; values"]</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr"/>
+          <t>["Music"]</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1031,65 +994,60 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Choosing a major;Research opportunities;Academics &amp; study habits;</t>
+          <t>Leadership &amp; military training;</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Systems Engineering;</t>
+          <t>Biology;</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Other;</t>
+          <t>Foreign language;None / undecided;</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Medical school;</t>
+          <t>PhD;</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Missiles;Public Affairs;</t>
+          <t>Weather;</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Not sure yet;Career military;</t>
+          <t>Medicine;</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Competition teams / clubs;</t>
+          <t>Summer research;Internships;Ops Air Force;</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Education;Climate / environment;</t>
+          <t>Ethics / philosophy;Aerospace / hypersonics;National security / policy;</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>I'm interested in Cold War nuclear strategy and hypersonic flow and heat shields.</t>
+          <t>I'm interested in Cold War nuclear strategy and human performance and sleep.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Hiking / outdoors;</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Global security;Ethics in technology;Healthcare;</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr"/>
+          <t>Cooking;Film / TV;Lifting;</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1109,65 +1067,60 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>["Academics &amp; study habits", "Grad school planning", "Research opportunities"]</t>
+          <t>["Leadership &amp; military training", "Wellness &amp; balance"]</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>["Operations Research"]</t>
+          <t>["Economics", "Behavioral Sciences"]</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>["Foreign language", "Other", "Nuclear Weapons &amp; Strategy"]</t>
+          <t>["Philosophy"]</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>["Medical school", "Marshall"]</t>
+          <t>["Gates Cambridge", "Law school", "Schwarzman"]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>["Scientist", "JAG", "Missiles"]</t>
+          <t>["Cyber", "JAG"]</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>["Medicine"]</t>
+          <t>["Government / policy"]</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>["Publishing research"]</t>
+          <t>["Jump", "Study abroad / exchange semester", "Summer research"]</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>["National security / policy", "Education", "Space"]</t>
+          <t>["Materials", "National security / policy", "Economics"]</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>I'm interested in leadership psychology under stress and ethics of autonomous weapons.</t>
+          <t>I'm interested in hypersonic flow and heat shields and Cold War nuclear strategy.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>["Faith community"]</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>["Climate", "Economic opportunity", "Mentorship / first-gen students"]</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr"/>
+          <t>["Cooking", "Team sports", "Film / TV"]</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1187,65 +1140,60 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Academics &amp; study habits;Wellness &amp; balance;</t>
+          <t>Time management;Wellness &amp; balance;Research opportunities;</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Humanities;Data Science;</t>
+          <t>Cyber Science;Mechanical Engineering;Political Science;</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Global Logistics;</t>
+          <t>Space Studies;</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Not sure yet;Law school;</t>
+          <t>Law school;Not sure yet;</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Missiles;RPA Pilot;</t>
+          <t>Intelligence;</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Industry / tech;</t>
+          <t>Not sure yet;Academia / research;Medicine;</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Competition teams / clubs;</t>
+          <t>Summer research;</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>National security / policy;</t>
+          <t>Education;Cybersecurity;</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>I'm interested in ethics of autonomous weapons and cyber defense of space systems.</t>
+          <t>I'm interested in ethics of autonomous weapons and leadership psychology under stress.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Running;Film / TV;Travel;</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Global security;Education access;Faith &amp; values;</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr"/>
+          <t>Travel;Cooking;</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1265,65 +1213,60 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>["Grad school planning", "Leadership &amp; military training", "Fellowships &amp; scholarships"]</t>
+          <t>["Grad school planning"]</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>["Political Science", "Meteorology"]</t>
+          <t>["Cyber Science"]</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>["Philosophy", "Other"]</t>
+          <t>["Space Studies", "Religion Studies"]</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>["Mitchell", "Hertz / NSF GRFP", "Not planning grad school"]</t>
+          <t>["Hertz / NSF GRFP"]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>["RPA Pilot", "Cyber", "Public Affairs"]</t>
+          <t>["Public Affairs", "Pilot", "Medical"]</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>["Career military"]</t>
+          <t>["Medicine", "Law", "Not sure yet"]</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>["Conferences / presenting"]</t>
+          <t>["Internships"]</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>["Cybersecurity", "Materials"]</t>
+          <t>["Biomedical / human performance", "Climate / environment"]</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>I'm interested in leadership psychology under stress and cyber defense of space systems.</t>
+          <t>I'm interested in machine learning for satellite imagery and quantum sensing.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>["Cooking", "Skiing / snowboarding", "Reading"]</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>["Veterans", "Mental health", "Faith &amp; values"]</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr"/>
+          <t>["Art / photography", "Climbing", "Faith community"]</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1343,65 +1286,60 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>26</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Fellowships &amp; scholarships;Navigating cadet life;Grad school planning;</t>
+          <t>Navigating cadet life;Choosing a major;</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Aeronautical Engineering;</t>
+          <t>Civil Engineering;Chemistry;Aeronautical Engineering;</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Space Studies;Religion Studies;</t>
+          <t>None / undecided;</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Truman;Not sure yet;PhD;</t>
+          <t>Fulbright;PhD;Not sure yet;</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Scientist;Weather;</t>
+          <t>Missiles;Space Operations;</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Academia / research;Career military;</t>
+          <t>Academia / research;Career military;Law;</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Jump;Competition teams / clubs;Cadet leadership positions;</t>
+          <t>Internships;Publishing research;Study abroad / exchange semester;</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Cybersecurity;Quantum / physics;Aerospace / hypersonics;</t>
+          <t>Biomedical / human performance;Economics;</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>I'm interested in great power competition and great power competition.</t>
+          <t>I'm interested in ethics of autonomous weapons and swarm autonomy for drones.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Travel;</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>Faith &amp; values;</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr"/>
+          <t>Music;Writing;</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1421,65 +1359,60 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>33</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>["Fellowships &amp; scholarships"]</t>
+          <t>["Wellness &amp; balance"]</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>["Humanities"]</t>
+          <t>["Data Science", "Management"]</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>["Philosophy", "Nuclear Weapons &amp; Strategy", "Foreign language"]</t>
+          <t>["Religion Studies", "Foreign language"]</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>["Medical school", "Master's right after graduation"]</t>
+          <t>["Gates Cambridge", "Hertz / NSF GRFP", "Medical school"]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>["Weather", "Medical", "Air Battle Manager"]</t>
+          <t>["JAG", "Security Forces", "Undecided"]</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>["Career military", "Industry / tech", "Law"]</t>
+          <t>["Academia / research"]</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>["Summer research", "Internships"]</t>
+          <t>["Publishing research", "Summer research", "Competition teams / clubs"]</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>["Psychology / leadership", "Quantum / physics", "AI / machine learning"]</t>
+          <t>["AI / machine learning"]</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>I'm interested in hypersonic flow and heat shields and cyber defense of space systems.</t>
+          <t>I'm interested in machine learning for satellite imagery and machine learning for satellite imagery.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>["Chess / board games", "Music"]</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>["Ethics in technology", "Healthcare", "Mentorship / first-gen students"]</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr"/>
+          <t>["Film / TV"]</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1499,65 +1432,60 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>40</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Time management;Grad school planning;</t>
+          <t>Choosing a major;Time management;Academics &amp; study habits;</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Legal Studies;Undecided;Data Science;</t>
+          <t>Military &amp; Strategic Studies;Legal Studies;</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Space Studies;Other;None / undecided;</t>
+          <t>None / undecided;Other;Foreign language;</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Mitchell;</t>
+          <t>Rhodes;Truman;Not sure yet;</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Maintenance / Logistics;</t>
+          <t>Combat Systems Officer;Air Battle Manager;</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Medicine;Career military;</t>
+          <t>Not sure yet;Entrepreneurship;Career military;</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Ops Air Force;Cadet leadership positions;Internships;</t>
+          <t>Competition teams / clubs;</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Materials;</t>
+          <t>Biomedical / human performance;History;</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>I'm interested in hypersonic flow and heat shields and machine learning for satellite imagery.</t>
+          <t>I'm interested in Cold War nuclear strategy and cyber defense of space systems.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Cooking;Skiing / snowboarding;Film / TV;</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>Healthcare;</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr"/>
+          <t>Film / TV;Gaming;Cooking;</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1577,65 +1505,60 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>["Choosing a major", "Navigating cadet life", "Leadership &amp; military training"]</t>
+          <t>["Time management", "Grad school planning"]</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>["Military &amp; Strategic Studies"]</t>
+          <t>["Chemistry", "Geospatial Science"]</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>["Religion Studies"]</t>
+          <t>["Other"]</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>["Mitchell", "Master's right after graduation", "Not planning grad school"]</t>
+          <t>["Gates Cambridge", "Marshall"]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>["Security Forces", "Intelligence"]</t>
+          <t>["Developmental Engineer", "Security Forces", "RPA Pilot"]</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>["Medicine", "Career military"]</t>
+          <t>["Entrepreneurship"]</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>["Jump", "Summer research", "Conferences / presenting"]</t>
+          <t>["Study abroad / exchange semester"]</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>["Psychology / leadership", "Climate / environment", "History"]</t>
+          <t>["History", "Aerospace / hypersonics", "Cybersecurity"]</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>I'm interested in swarm autonomy for drones and quantum sensing.</t>
+          <t>I'm interested in machine learning for satellite imagery and cyber defense of space systems.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>["Chess / board games", "Writing"]</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>["Education access", "Economic opportunity", "Climate"]</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr"/>
+          <t>["Hiking / outdoors"]</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1655,65 +1578,60 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>AF/SF career planning;</t>
+          <t>Fellowships &amp; scholarships;Grad school planning;</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Astronautical Engineering;Undecided;</t>
+          <t>Operations Research;</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Nuclear Weapons &amp; Strategy;</t>
+          <t>Other;Religion Studies;</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Not planning grad school;</t>
+          <t>Truman;Gates Cambridge;</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Scientist;Maintenance / Logistics;</t>
+          <t>RPA Pilot;Missiles;</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Not sure yet;</t>
+          <t>Medicine;</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Jump;Internships;Soaring / powered flight;</t>
+          <t>Competition teams / clubs;Conferences / presenting;Summer research;</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Energy;</t>
+          <t>National security / policy;Quantum / physics;</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>I'm interested in quantum sensing and hypersonic flow and heat shields.</t>
+          <t>I'm interested in leadership psychology under stress and Cold War nuclear strategy.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Running;Climbing;</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>Education access;Faith &amp; values;</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr"/>
+          <t>Climbing;Hiking / outdoors;Travel;</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1738,60 +1656,55 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>["AF/SF career planning"]</t>
+          <t>["Choosing a major"]</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>["History"]</t>
+          <t>["Data Science", "Astronautical Engineering"]</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>["Global Logistics"]</t>
+          <t>["Nuclear Weapons &amp; Strategy"]</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>["Mitchell", "Schwarzman", "PhD"]</t>
+          <t>["Not planning grad school"]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>["Combat Systems Officer"]</t>
+          <t>["Scientist", "Maintenance / Logistics"]</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>["Government / policy", "Career military", "Industry / tech"]</t>
+          <t>["Not sure yet"]</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>["Summer research", "Study abroad / exchange semester"]</t>
+          <t>["Jump", "Internships", "Soaring / powered flight"]</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>["Materials"]</t>
+          <t>["Energy"]</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>I'm interested in renewable energy on bases and Cold War nuclear strategy.</t>
+          <t>I'm interested in quantum sensing and hypersonic flow and heat shields.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>["Music", "Writing", "Gaming"]</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>["Economic opportunity", "Veterans", "Ethics in technology"]</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr"/>
+          <t>["Running", "Climbing"]</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1811,65 +1724,60 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>AF/SF career planning;</t>
+          <t>Wellness &amp; balance;</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Aeronautical Engineering;</t>
+          <t>Behavioral Sciences;</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Space Studies;</t>
+          <t>Philosophy;Space Studies;</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Hertz / NSF GRFP;Truman;Not planning grad school;</t>
+          <t>Gates Cambridge;</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Undecided;</t>
+          <t>Security Forces;Scientist;Space Operations;</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Not sure yet;Entrepreneurship;</t>
+          <t>Government / policy;</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Publishing research;Soaring / powered flight;</t>
+          <t>Study abroad / exchange semester;</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Biomedical / human performance;Space;Energy;</t>
+          <t>Autonomy / drones;Aerospace / hypersonics;</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>I'm interested in ethics of autonomous weapons and renewable energy on bases.</t>
+          <t>I'm interested in ethics of autonomous weapons and Cold War nuclear strategy.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Faith community;</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>Mental health;Veterans;</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr"/>
+          <t>Writing;Music;Skiing / snowboarding;</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1889,65 +1797,60 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>29</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>["AF/SF career planning"]</t>
+          <t>["Fellowships &amp; scholarships", "AF/SF career planning", "Research opportunities"]</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>["Civil Engineering", "Astronautical Engineering"]</t>
+          <t>["Data Science"]</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>["Other"]</t>
+          <t>["Foreign language"]</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>["Medical school", "Schwarzman", "PhD"]</t>
+          <t>["Law school"]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>["Acquisitions / Program Management"]</t>
+          <t>["Weather", "Intelligence", "JAG"]</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>["Not sure yet"]</t>
+          <t>["Government / policy", "Not sure yet"]</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>["Study abroad / exchange semester"]</t>
+          <t>["Cadet leadership positions"]</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>["Psychology / leadership", "AI / machine learning"]</t>
+          <t>["Education", "Quantum / physics", "Economics"]</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>I'm interested in Cold War nuclear strategy and human performance and sleep.</t>
+          <t>I'm interested in quantum sensing and great power competition.</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>["Art / photography", "Gaming"]</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>["Ethics in technology"]</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr"/>
+          <t>["Music", "Gaming"]</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1967,65 +1870,60 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fellowships &amp; scholarships;Academics &amp; study habits;</t>
+          <t>Fellowships &amp; scholarships;</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Foreign Area Studies;Behavioral Sciences;</t>
+          <t>English;Astronautical Engineering;</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Nuclear Weapons &amp; Strategy;None / undecided;</t>
+          <t>Foreign language;</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Truman;Not planning grad school;Master's right after graduation;</t>
+          <t>Medical school;</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>RPA Pilot;</t>
+          <t>Scientist;Security Forces;Cyber;</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Industry / tech;Not sure yet;</t>
+          <t>Industry / tech;</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Conferences / presenting;Summer research;</t>
+          <t>Cadet leadership positions;Publishing research;Soaring / powered flight;</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>AI / machine learning;Cybersecurity;</t>
+          <t>Climate / environment;History;Cybersecurity;</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>I'm interested in Cold War nuclear strategy and renewable energy on bases.</t>
+          <t>I'm interested in swarm autonomy for drones and cyber defense of space systems.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Climbing;</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>Mentorship / first-gen students;Veterans;Community service;</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr"/>
+          <t>Team sports;</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2045,65 +1943,60 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>18</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>["Leadership &amp; military training", "Fellowships &amp; scholarships", "AF/SF career planning"]</t>
+          <t>["Academics &amp; study habits", "AF/SF career planning"]</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>["Mechanical Engineering", "Meteorology", "Chemistry"]</t>
+          <t>["Electrical &amp; Computer Engineering", "Management"]</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>["Other"]</t>
+          <t>["Space Studies", "Foreign language"]</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>["Law school", "Not sure yet", "Master's right after graduation"]</t>
+          <t>["Truman", "Gates Cambridge"]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>["JAG"]</t>
+          <t>["Pilot"]</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>["Career military", "Law", "Medicine"]</t>
+          <t>["Law", "Career military"]</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>["Ops Air Force", "Internships", "Summer research"]</t>
+          <t>["Soaring / powered flight", "Publishing research"]</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>["Cybersecurity"]</t>
+          <t>["Biomedical / human performance", "Space", "Quantum / physics"]</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>I'm interested in renewable energy on bases and human performance and sleep.</t>
+          <t>I'm interested in swarm autonomy for drones and hypersonic flow and heat shields.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>["Faith community"]</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>["Mentorship / first-gen students", "Mental health"]</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr"/>
+          <t>["Climbing", "Skiing / snowboarding"]</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2123,17 +2016,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>26</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Time management;Grad school planning;Leadership &amp; military training;</t>
+          <t>Academics &amp; study habits;Navigating cadet life;Wellness &amp; balance;</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Aeronautical Engineering;History;</t>
+          <t>Economics;Meteorology;</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2143,45 +2036,40 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Master's right after graduation;Marshall;Law school;</t>
+          <t>Master's right after graduation;Not sure yet;Fulbright;</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Medical;Scientist;RPA Pilot;</t>
+          <t>Public Affairs;Maintenance / Logistics;Special Warfare;</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Government / policy;Medicine;</t>
+          <t>Not sure yet;Industry / tech;Academia / research;</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Ops Air Force;</t>
+          <t>Conferences / presenting;Study abroad / exchange semester;Summer research;</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Psychology / leadership;Climate / environment;Economics;</t>
+          <t>Economics;History;Psychology / leadership;</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>I'm interested in quantum sensing and hypersonic flow and heat shields.</t>
+          <t>I'm interested in great power competition and machine learning for satellite imagery.</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Writing;Lifting;</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>Economic opportunity;Climate;Education access;</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr"/>
+          <t>Chess / board games;Running;Volunteering;</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2201,65 +2089,60 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>38</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>["Research opportunities"]</t>
+          <t>["Grad school planning", "Choosing a major", "Academics &amp; study habits"]</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>["Meteorology", "Philosophy"]</t>
+          <t>["Chemistry"]</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>["Nuclear Weapons &amp; Strategy", "None / undecided", "Other"]</t>
+          <t>["Global Logistics", "Foreign language", "Space Studies"]</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>["Rhodes"]</t>
+          <t>["Master's right after graduation", "Rhodes"]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>["Combat Systems Officer", "Medical"]</t>
+          <t>["Pilot", "Weather", "Developmental Engineer"]</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>["Industry / tech", "Medicine"]</t>
+          <t>["Entrepreneurship", "Career military"]</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>["Competition teams / clubs"]</t>
+          <t>["Internships", "Publishing research"]</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>["Materials", "Climate / environment"]</t>
+          <t>["Aerospace / hypersonics", "National security / policy", "Quantum / physics"]</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>I'm interested in cyber defense of space systems and cyber defense of space systems.</t>
+          <t>I'm interested in hypersonic flow and heat shields and cyber defense of space systems.</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>["Music"]</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>["Education access", "Healthcare"]</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr"/>
+          <t>["Climbing", "Reading"]</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2279,65 +2162,60 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Leadership &amp; military training;Choosing a major;</t>
+          <t>Grad school planning;Wellness &amp; balance;Leadership &amp; military training;</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>History;Data Science;Foreign Area Studies;</t>
+          <t>Systems Engineering;Foreign Area Studies;</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Space Studies;</t>
+          <t>None / undecided;</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>PhD;</t>
+          <t>Schwarzman;Not sure yet;Rhodes;</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Space Operations;</t>
+          <t>Undecided;Intelligence;RPA Pilot;</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Entrepreneurship;Academia / research;Industry / tech;</t>
+          <t>Academia / research;Not sure yet;Law;</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Publishing research;Soaring / powered flight;Internships;</t>
+          <t>Soaring / powered flight;Study abroad / exchange semester;Summer research;</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>History;Space;Climate / environment;</t>
+          <t>Autonomy / drones;Climate / environment;</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>I'm interested in cyber defense of space systems and quantum sensing.</t>
+          <t>I'm interested in Cold War nuclear strategy and renewable energy on bases.</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Team sports;</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>Healthcare;</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr"/>
+          <t>Music;</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2357,65 +2235,60 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>32</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>["AF/SF career planning", "Fellowships &amp; scholarships"]</t>
+          <t>["Time management", "AF/SF career planning"]</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>["English", "Foreign Area Studies"]</t>
+          <t>["History", "Physics"]</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>["Philosophy", "Other"]</t>
+          <t>["Space Studies"]</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>["Rhodes", "Gates Cambridge"]</t>
+          <t>["Marshall", "Hertz / NSF GRFP"]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>["Maintenance / Logistics", "Air Battle Manager"]</t>
+          <t>["Acquisitions / Program Management"]</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>["Career military"]</t>
+          <t>["Industry / tech", "Law"]</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>["Soaring / powered flight", "Conferences / presenting", "Jump"]</t>
+          <t>["Competition teams / clubs", "Soaring / powered flight", "Cadet leadership positions"]</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>["Ethics / philosophy"]</t>
+          <t>["Biomedical / human performance"]</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>I'm interested in quantum sensing and leadership psychology under stress.</t>
+          <t>I'm interested in hypersonic flow and heat shields and leadership psychology under stress.</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>["Cooking"]</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>["Ethics in technology", "Mental health"]</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr"/>
+          <t>["Skiing / snowboarding"]</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2435,65 +2308,60 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Academics &amp; study habits;</t>
+          <t>Research opportunities;Fellowships &amp; scholarships;</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Economics;Meteorology;Chemistry;</t>
+          <t>Space Operations;Meteorology;Legal Studies;</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Nuclear Weapons &amp; Strategy;</t>
+          <t>Philosophy;Global Logistics;</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Master's right after graduation;Gates Cambridge;</t>
+          <t>Truman;Hertz / NSF GRFP;</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Missiles;</t>
+          <t>Maintenance / Logistics;Pilot;</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Career military;Law;</t>
+          <t>Career military;</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Cadet leadership positions;Publishing research;Ops Air Force;</t>
+          <t>Competition teams / clubs;Cadet leadership positions;</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Aerospace / hypersonics;AI / machine learning;History;</t>
+          <t>Cybersecurity;Biomedical / human performance;</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>I'm interested in quantum sensing and cyber defense of space systems.</t>
+          <t>I'm interested in human performance and sleep and quantum sensing.</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Skiing / snowboarding;Writing;Gaming;</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>Mentorship / first-gen students;</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr"/>
+          <t>Hiking / outdoors;Art / photography;</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2513,65 +2381,60 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>["Leadership &amp; military training"]</t>
+          <t>["Research opportunities", "Navigating cadet life"]</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>["Electrical &amp; Computer Engineering", "Economics"]</t>
+          <t>["Computer Science"]</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>["Nuclear Weapons &amp; Strategy", "Global Logistics"]</t>
+          <t>["Foreign language", "Global Logistics", "Religion Studies"]</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>["Medical school", "Schwarzman", "Mitchell"]</t>
+          <t>["Gates Cambridge", "Marshall"]</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>["Developmental Engineer", "Acquisitions / Program Management", "Medical"]</t>
+          <t>["Maintenance / Logistics", "Finance / Contracting"]</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>["Law", "Career military", "Industry / tech"]</t>
+          <t>["Medicine"]</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>["Study abroad / exchange semester", "Internships", "Ops Air Force"]</t>
+          <t>["Soaring / powered flight", "Summer research"]</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>["Education", "Quantum / physics", "Space"]</t>
+          <t>["Space", "AI / machine learning"]</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>I'm interested in cyber defense of space systems and human performance and sleep.</t>
+          <t>I'm interested in renewable energy on bases and Cold War nuclear strategy.</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>["Volunteering", "Skiing / snowboarding"]</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>["Climate", "Economic opportunity", "Education access"]</t>
-        </is>
-      </c>
-      <c r="P27" t="inlineStr"/>
+          <t>["Skiing / snowboarding", "Gaming", "Chess / board games"]</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2591,65 +2454,60 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>28</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Time management;Choosing a major;</t>
+          <t>Research opportunities;Grad school planning;Wellness &amp; balance;</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Cyber Science;English;</t>
+          <t>Undecided;Aeronautical Engineering;</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Space Studies;Foreign language;</t>
+          <t>Other;Nuclear Weapons &amp; Strategy;None / undecided;</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Not planning grad school;Mitchell;Not sure yet;</t>
+          <t>Law school;</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>JAG;Intelligence;</t>
+          <t>Combat Systems Officer;</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Entrepreneurship;Academia / research;</t>
+          <t>Law;Government / policy;Entrepreneurship;</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Competition teams / clubs;</t>
+          <t>Soaring / powered flight;</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>History;Aerospace / hypersonics;</t>
+          <t>Autonomy / drones;Psychology / leadership;</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>I'm interested in renewable energy on bases and great power competition.</t>
+          <t>I'm interested in great power competition and machine learning for satellite imagery.</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Music;Climbing;Skiing / snowboarding;</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>Community service;</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr"/>
+          <t>Film / TV;</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2669,65 +2527,60 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>["Leadership &amp; military training", "Navigating cadet life", "AF/SF career planning"]</t>
+          <t>["AF/SF career planning", "Wellness &amp; balance"]</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>["Chemistry"]</t>
+          <t>["Philosophy", "Meteorology"]</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>["Other"]</t>
+          <t>["Other", "Global Logistics"]</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>["Not sure yet", "Not planning grad school", "Hertz / NSF GRFP"]</t>
+          <t>["Schwarzman"]</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>["Medical", "Pilot", "RPA Pilot"]</t>
+          <t>["Weather", "Maintenance / Logistics"]</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>["Not sure yet", "Government / policy"]</t>
+          <t>["Academia / research"]</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>["Internships"]</t>
+          <t>["Study abroad / exchange semester", "Internships", "Ops Air Force"]</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>["Cybersecurity"]</t>
+          <t>["Education", "Quantum / physics", "Space"]</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>I'm interested in machine learning for satellite imagery and great power competition.</t>
+          <t>I'm interested in cyber defense of space systems and human performance and sleep.</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>["Hiking / outdoors", "Travel", "Lifting"]</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>["Mental health", "Economic opportunity", "Veterans"]</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr"/>
+          <t>["Volunteering", "Skiing / snowboarding"]</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Form feedback: focus up to 5, NGO/nonprofit, not-interested-in-research
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Martinson_Matching_SAMPLE.xlsx
+++ b/Martinson_Matching_SAMPLE.xlsx
@@ -659,7 +659,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>["Academia / research", "Career military", "Entrepreneurship"]</t>
+          <t>["Academia / research", "Industry / tech", "Entrepreneurship"]</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -669,17 +669,17 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>["Aerospace / hypersonics", "Materials", "AI / machine learning"]</t>
+          <t>["Aerospace / hypersonics", "Autonomy / drones", "Materials"]</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>I'm interested in leadership psychology under stress and ethics of autonomous weapons.</t>
+          <t>I'm interested in ethics of autonomous weapons and cyber defense of space systems.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>["Volunteering", "Art / photography"]</t>
+          <t>["Volunteering", "Art / photography", "Gaming"]</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -702,12 +702,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>38</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Leadership &amp; military training;Research opportunities;AF/SF career planning;</t>
+          <t>Research opportunities;AF/SF career planning;</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Not sure yet;Academia / research;</t>
+          <t>NGO / nonprofit;Entrepreneurship;</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -805,27 +805,27 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>["Entrepreneurship", "Medicine", "Not sure yet"]</t>
+          <t>["Entrepreneurship", "NGO / nonprofit", "Academia / research"]</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>["Competition teams / clubs", "Soaring / powered flight", "Cadet leadership positions"]</t>
+          <t>["Cadet leadership positions", "Jump", "Summer research"]</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>["History", "AI / machine learning", "Climate / environment"]</t>
+          <t>["History", "Energy"]</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>I'm interested in human performance and sleep and machine learning for satellite imagery.</t>
+          <t>I'm interested in leadership psychology under stress and hypersonic flow and heat shields.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>["Hiking / outdoors", "Film / TV", "Running"]</t>
+          <t>["Lifting", "Music"]</t>
         </is>
       </c>
       <c r="O5" t="inlineStr"/>
@@ -848,12 +848,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Fellowships &amp; scholarships;Grad school planning;</t>
+          <t>Grad school planning;</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -878,27 +878,27 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Entrepreneurship;Medicine;Government / policy;</t>
+          <t>Entrepreneurship;Law;Academia / research;</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Cadet leadership positions;Ops Air Force;</t>
+          <t>Cadet leadership positions;Ops Air Force;Study abroad / exchange semester;</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Aerospace / hypersonics;</t>
+          <t>Energy;</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>I'm interested in machine learning for satellite imagery and machine learning for satellite imagery.</t>
+          <t>I'm interested in machine learning for satellite imagery and ethics of autonomous weapons.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Gaming;</t>
+          <t>Gaming;Running;Chess / board games;</t>
         </is>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -921,57 +921,57 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>38</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>["Wellness &amp; balance", "Fellowships &amp; scholarships"]</t>
+          <t>["AF/SF career planning"]</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>["Economics", "Aeronautical Engineering"]</t>
+          <t>["Aeronautical Engineering", "Chemistry"]</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["Other"]</t>
+          <t>["Global Logistics", "Nuclear Weapons &amp; Strategy"]</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>["Gates Cambridge", "PhD", "Not sure yet"]</t>
+          <t>["Gates Cambridge", "Fulbright", "Law school"]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>["Space Operations", "JAG"]</t>
+          <t>["Public Affairs", "Combat Systems Officer", "OSI"]</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>["Career military", "Government / policy", "Medicine"]</t>
+          <t>["Not sure yet", "Law", "Government / policy"]</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>["Cadet leadership positions", "Conferences / presenting", "Publishing research"]</t>
+          <t>["Cadet leadership positions", "Internships"]</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>["Space", "Climate / environment"]</t>
+          <t>["Ethics / philosophy", "Autonomy / drones"]</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>I'm interested in renewable energy on bases and quantum sensing.</t>
+          <t>I'm interested in ethics of autonomous weapons and hypersonic flow and heat shields.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>["Music"]</t>
+          <t>["Travel"]</t>
         </is>
       </c>
       <c r="O7" t="inlineStr"/>
@@ -994,57 +994,57 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Leadership &amp; military training;</t>
+          <t>Research opportunities;</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Biology;</t>
+          <t>Astronautical Engineering;Biology;Aeronautical Engineering;</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Foreign language;None / undecided;</t>
+          <t>Religion Studies;Nuclear Weapons &amp; Strategy;Foreign language;</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>PhD;</t>
+          <t>PhD;Rhodes;</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Weather;</t>
+          <t>Intelligence;</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Medicine;</t>
+          <t>Law;Academia / research;Medicine;</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Summer research;Internships;Ops Air Force;</t>
+          <t>Jump;Conferences / presenting;</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Ethics / philosophy;Aerospace / hypersonics;National security / policy;</t>
+          <t>Space;Not interested in research;</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>I'm interested in Cold War nuclear strategy and human performance and sleep.</t>
+          <t>I'm interested in cyber defense of space systems and cyber defense of space systems.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Cooking;Film / TV;Lifting;</t>
+          <t>Film / TV;Writing;</t>
         </is>
       </c>
       <c r="O8" t="inlineStr"/>
@@ -1067,57 +1067,57 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>["Leadership &amp; military training", "Wellness &amp; balance"]</t>
+          <t>["Choosing a major"]</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>["Economics", "Behavioral Sciences"]</t>
+          <t>["Electrical &amp; Computer Engineering", "Philosophy", "Data Science"]</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>["Philosophy"]</t>
+          <t>["Religion Studies", "Nuclear Weapons &amp; Strategy"]</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>["Gates Cambridge", "Law school", "Schwarzman"]</t>
+          <t>["Truman"]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>["Cyber", "JAG"]</t>
+          <t>["Missiles", "Space Operations", "Weather"]</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>["Government / policy"]</t>
+          <t>["Not sure yet"]</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>["Jump", "Study abroad / exchange semester", "Summer research"]</t>
+          <t>["Internships", "Soaring / powered flight"]</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>["Materials", "National security / policy", "Economics"]</t>
+          <t>["History", "Energy", "Education"]</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>I'm interested in hypersonic flow and heat shields and Cold War nuclear strategy.</t>
+          <t>I'm interested in ethics of autonomous weapons and great power competition.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>["Cooking", "Team sports", "Film / TV"]</t>
+          <t>["Chess / board games", "Art / photography", "Film / TV"]</t>
         </is>
       </c>
       <c r="O9" t="inlineStr"/>
@@ -1145,52 +1145,52 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Time management;Wellness &amp; balance;Research opportunities;</t>
+          <t>Grad school planning;Wellness &amp; balance;Navigating cadet life;</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Cyber Science;Mechanical Engineering;Political Science;</t>
+          <t>Political Science;Cyber Science;Computer Science;</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Space Studies;</t>
+          <t>None / undecided;Religion Studies;Global Logistics;</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Law school;Not sure yet;</t>
+          <t>Rhodes;</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Intelligence;</t>
+          <t>Medical;Scientist;</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Not sure yet;Academia / research;Medicine;</t>
+          <t>Medicine;</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Summer research;</t>
+          <t>Jump;Conferences / presenting;</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Education;Cybersecurity;</t>
+          <t>Climate / environment;</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>I'm interested in ethics of autonomous weapons and leadership psychology under stress.</t>
+          <t>I'm interested in hypersonic flow and heat shields and ethics of autonomous weapons.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Travel;Cooking;</t>
+          <t>Music;Art / photography;</t>
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -1213,57 +1213,57 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>["Grad school planning"]</t>
+          <t>["Wellness &amp; balance", "Academics &amp; study habits"]</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>["Cyber Science"]</t>
+          <t>["Meteorology", "English"]</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>["Space Studies", "Religion Studies"]</t>
+          <t>["Philosophy", "Other", "Global Logistics"]</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>["Hertz / NSF GRFP"]</t>
+          <t>["Mitchell"]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>["Public Affairs", "Pilot", "Medical"]</t>
+          <t>["Intelligence", "Medical", "Cyber"]</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>["Medicine", "Law", "Not sure yet"]</t>
+          <t>["Medicine", "Industry / tech"]</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>["Internships"]</t>
+          <t>["Cadet leadership positions", "Competition teams / clubs", "Conferences / presenting"]</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>["Biomedical / human performance", "Climate / environment"]</t>
+          <t>["Aerospace / hypersonics", "Energy", "Not interested in research"]</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>I'm interested in machine learning for satellite imagery and quantum sensing.</t>
+          <t>I'm interested in machine learning for satellite imagery and swarm autonomy for drones.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>["Art / photography", "Climbing", "Faith community"]</t>
+          <t>["Travel"]</t>
         </is>
       </c>
       <c r="O11" t="inlineStr"/>
@@ -1286,57 +1286,57 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Navigating cadet life;Choosing a major;</t>
+          <t>Wellness &amp; balance;Leadership &amp; military training;Research opportunities;</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Civil Engineering;Chemistry;Aeronautical Engineering;</t>
+          <t>Management;</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>None / undecided;</t>
+          <t>Religion Studies;Foreign language;Other;</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Fulbright;PhD;Not sure yet;</t>
+          <t>Medical school;Marshall;Master's right after graduation;</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Missiles;Space Operations;</t>
+          <t>Space Operations;Security Forces;Intelligence;</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Academia / research;Career military;Law;</t>
+          <t>Career military;</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Internships;Publishing research;Study abroad / exchange semester;</t>
+          <t>Ops Air Force;Soaring / powered flight;</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Biomedical / human performance;Economics;</t>
+          <t>Climate / environment;National security / policy;Cybersecurity;</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>I'm interested in ethics of autonomous weapons and swarm autonomy for drones.</t>
+          <t>I'm interested in great power competition and quantum sensing.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Music;Writing;</t>
+          <t>Lifting;</t>
         </is>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -1359,32 +1359,32 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>["Wellness &amp; balance"]</t>
+          <t>["Wellness &amp; balance", "Time management"]</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>["Data Science", "Management"]</t>
+          <t>["Space Operations", "Undecided"]</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>["Religion Studies", "Foreign language"]</t>
+          <t>["Religion Studies", "Nuclear Weapons &amp; Strategy", "Philosophy"]</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>["Gates Cambridge", "Hertz / NSF GRFP", "Medical school"]</t>
+          <t>["Master's right after graduation", "Rhodes", "Hertz / NSF GRFP"]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>["JAG", "Security Forces", "Undecided"]</t>
+          <t>["Public Affairs"]</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1394,22 +1394,22 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>["Publishing research", "Summer research", "Competition teams / clubs"]</t>
+          <t>["Study abroad / exchange semester"]</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>["AI / machine learning"]</t>
+          <t>["Space", "Autonomy / drones"]</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>I'm interested in machine learning for satellite imagery and machine learning for satellite imagery.</t>
+          <t>I'm interested in human performance and sleep and renewable energy on bases.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>["Film / TV"]</t>
+          <t>["Chess / board games", "Film / TV", "Faith community"]</t>
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -1432,57 +1432,57 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Choosing a major;Time management;Academics &amp; study habits;</t>
+          <t>Academics &amp; study habits;Grad school planning;Time management;</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Military &amp; Strategic Studies;Legal Studies;</t>
+          <t>Astronautical Engineering;Physics;</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>None / undecided;Other;Foreign language;</t>
+          <t>None / undecided;</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Rhodes;Truman;Not sure yet;</t>
+          <t>Rhodes;Not sure yet;Marshall;</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Combat Systems Officer;Air Battle Manager;</t>
+          <t>Special Warfare;Public Affairs;</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Not sure yet;Entrepreneurship;Career military;</t>
+          <t>Not sure yet;Government / policy;Medicine;</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Competition teams / clubs;</t>
+          <t>Competition teams / clubs;Publishing research;</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Biomedical / human performance;History;</t>
+          <t>Education;Climate / environment;History;</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>I'm interested in Cold War nuclear strategy and cyber defense of space systems.</t>
+          <t>I'm interested in great power competition and Cold War nuclear strategy.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Film / TV;Gaming;Cooking;</t>
+          <t>Music;Travel;Climbing;</t>
         </is>
       </c>
       <c r="O14" t="inlineStr"/>
@@ -1505,57 +1505,57 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>["Time management", "Grad school planning"]</t>
+          <t>["Navigating cadet life"]</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>["Chemistry", "Geospatial Science"]</t>
+          <t>["Electrical &amp; Computer Engineering", "Behavioral Sciences"]</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>["Other"]</t>
+          <t>["Space Studies", "None / undecided", "Foreign language"]</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>["Gates Cambridge", "Marshall"]</t>
+          <t>["Medical school"]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>["Developmental Engineer", "Security Forces", "RPA Pilot"]</t>
+          <t>["Air Battle Manager", "Space Operations"]</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>["Entrepreneurship"]</t>
+          <t>["Medicine", "Academia / research", "NGO / nonprofit"]</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>["Study abroad / exchange semester"]</t>
+          <t>["Competition teams / clubs"]</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>["History", "Aerospace / hypersonics", "Cybersecurity"]</t>
+          <t>["Space"]</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>I'm interested in machine learning for satellite imagery and cyber defense of space systems.</t>
+          <t>I'm interested in quantum sensing and cyber defense of space systems.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>["Hiking / outdoors"]</t>
+          <t>["Gaming"]</t>
         </is>
       </c>
       <c r="O15" t="inlineStr"/>
@@ -1578,57 +1578,57 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Fellowships &amp; scholarships;Grad school planning;</t>
+          <t>Navigating cadet life;Time management;Wellness &amp; balance;</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Operations Research;</t>
+          <t>Geospatial Science;Computer Science;</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Other;Religion Studies;</t>
+          <t>Global Logistics;Foreign language;</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Truman;Gates Cambridge;</t>
+          <t>Gates Cambridge;Rhodes;Not planning grad school;</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>RPA Pilot;Missiles;</t>
+          <t>OSI;Undecided;Pilot;</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Medicine;</t>
+          <t>Medicine;Entrepreneurship;</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Competition teams / clubs;Conferences / presenting;Summer research;</t>
+          <t>Internships;Conferences / presenting;Ops Air Force;</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>National security / policy;Quantum / physics;</t>
+          <t>Aerospace / hypersonics;</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>I'm interested in leadership psychology under stress and Cold War nuclear strategy.</t>
+          <t>I'm interested in Cold War nuclear strategy and Cold War nuclear strategy.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Climbing;Hiking / outdoors;Travel;</t>
+          <t>Team sports;</t>
         </is>
       </c>
       <c r="O16" t="inlineStr"/>
@@ -1651,57 +1651,57 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>18</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>["Choosing a major"]</t>
+          <t>["Navigating cadet life"]</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>["Data Science", "Astronautical Engineering"]</t>
+          <t>["Space Operations", "Data Science", "Foreign Area Studies"]</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>["Nuclear Weapons &amp; Strategy"]</t>
+          <t>["None / undecided"]</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>["Not planning grad school"]</t>
+          <t>["Gates Cambridge", "Marshall", "Schwarzman"]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>["Scientist", "Maintenance / Logistics"]</t>
+          <t>["Cyber"]</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>["Not sure yet"]</t>
+          <t>["Industry / tech", "Entrepreneurship"]</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>["Jump", "Internships", "Soaring / powered flight"]</t>
+          <t>["Internships"]</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>["Energy"]</t>
+          <t>["Aerospace / hypersonics", "Climate / environment"]</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>I'm interested in quantum sensing and hypersonic flow and heat shields.</t>
+          <t>I'm interested in hypersonic flow and heat shields and Cold War nuclear strategy.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>["Running", "Climbing"]</t>
+          <t>["Travel"]</t>
         </is>
       </c>
       <c r="O17" t="inlineStr"/>
@@ -1724,57 +1724,57 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Wellness &amp; balance;</t>
+          <t>Time management;Navigating cadet life;</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Behavioral Sciences;</t>
+          <t>Mechanical Engineering;Chemistry;</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Philosophy;Space Studies;</t>
+          <t>Space Studies;</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Gates Cambridge;</t>
+          <t>Fulbright;</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Security Forces;Scientist;Space Operations;</t>
+          <t>Combat Systems Officer;Cyber;</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Government / policy;</t>
+          <t>Entrepreneurship;</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Study abroad / exchange semester;</t>
+          <t>Soaring / powered flight;Publishing research;Ops Air Force;</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Autonomy / drones;Aerospace / hypersonics;</t>
+          <t>Psychology / leadership;Energy;</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>I'm interested in ethics of autonomous weapons and Cold War nuclear strategy.</t>
+          <t>I'm interested in Cold War nuclear strategy and human performance and sleep.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Writing;Music;Skiing / snowboarding;</t>
+          <t>Reading;</t>
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
@@ -1797,57 +1797,57 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>["Fellowships &amp; scholarships", "AF/SF career planning", "Research opportunities"]</t>
+          <t>["Academics &amp; study habits"]</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>["Data Science"]</t>
+          <t>["Legal Studies", "Management", "Computer Science"]</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>["Foreign language"]</t>
+          <t>["None / undecided", "Philosophy", "Space Studies"]</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>["Law school"]</t>
+          <t>["Medical school"]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>["Weather", "Intelligence", "JAG"]</t>
+          <t>["Security Forces", "Medical", "Weather"]</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>["Government / policy", "Not sure yet"]</t>
+          <t>["Not sure yet", "Entrepreneurship"]</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>["Cadet leadership positions"]</t>
+          <t>["Ops Air Force", "Conferences / presenting", "Jump"]</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>["Education", "Quantum / physics", "Economics"]</t>
+          <t>["Cybersecurity"]</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>I'm interested in quantum sensing and great power competition.</t>
+          <t>I'm interested in quantum sensing and human performance and sleep.</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>["Music", "Gaming"]</t>
+          <t>["Skiing / snowboarding"]</t>
         </is>
       </c>
       <c r="O19" t="inlineStr"/>
@@ -1870,57 +1870,57 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fellowships &amp; scholarships;</t>
+          <t>AF/SF career planning;</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>English;Astronautical Engineering;</t>
+          <t>Civil Engineering;Astronautical Engineering;</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Foreign language;</t>
+          <t>Other;</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Medical school;</t>
+          <t>Medical school;Schwarzman;PhD;</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Scientist;Security Forces;Cyber;</t>
+          <t>Acquisitions / Program Management;</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Industry / tech;</t>
+          <t>NGO / nonprofit;</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Cadet leadership positions;Publishing research;Soaring / powered flight;</t>
+          <t>Study abroad / exchange semester;</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Climate / environment;History;Cybersecurity;</t>
+          <t>Psychology / leadership;AI / machine learning;</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>I'm interested in swarm autonomy for drones and cyber defense of space systems.</t>
+          <t>I'm interested in Cold War nuclear strategy and human performance and sleep.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Team sports;</t>
+          <t>Art / photography;Gaming;</t>
         </is>
       </c>
       <c r="O20" t="inlineStr"/>
@@ -1943,57 +1943,57 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>["Academics &amp; study habits", "AF/SF career planning"]</t>
+          <t>["Grad school planning", "Research opportunities"]</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>["Electrical &amp; Computer Engineering", "Management"]</t>
+          <t>["Aeronautical Engineering"]</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>["Space Studies", "Foreign language"]</t>
+          <t>["Other", "Foreign language"]</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>["Truman", "Gates Cambridge"]</t>
+          <t>["Schwarzman", "Master's right after graduation"]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>["Pilot"]</t>
+          <t>["Intelligence", "Developmental Engineer", "JAG"]</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>["Law", "Career military"]</t>
+          <t>["Industry / tech"]</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>["Soaring / powered flight", "Publishing research"]</t>
+          <t>["Internships", "Study abroad / exchange semester"]</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>["Biomedical / human performance", "Space", "Quantum / physics"]</t>
+          <t>["Autonomy / drones", "Ethics / philosophy"]</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>I'm interested in swarm autonomy for drones and hypersonic flow and heat shields.</t>
+          <t>I'm interested in swarm autonomy for drones and Cold War nuclear strategy.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>["Climbing", "Skiing / snowboarding"]</t>
+          <t>["Gaming", "Climbing"]</t>
         </is>
       </c>
       <c r="O21" t="inlineStr"/>
@@ -2016,57 +2016,57 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>38</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Academics &amp; study habits;Navigating cadet life;Wellness &amp; balance;</t>
+          <t>Fellowships &amp; scholarships;Navigating cadet life;Research opportunities;</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Economics;Meteorology;</t>
+          <t>Humanities;Chemistry;Economics;</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Philosophy;</t>
+          <t>Religion Studies;Foreign language;Global Logistics;</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Master's right after graduation;Not sure yet;Fulbright;</t>
+          <t>Medical school;Mitchell;Law school;</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Public Affairs;Maintenance / Logistics;Special Warfare;</t>
+          <t>JAG;Space Operations;Undecided;</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Not sure yet;Industry / tech;Academia / research;</t>
+          <t>Career military;Government / policy;Not sure yet;</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Conferences / presenting;Study abroad / exchange semester;Summer research;</t>
+          <t>Summer research;</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Economics;History;Psychology / leadership;</t>
+          <t>History;</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>I'm interested in great power competition and machine learning for satellite imagery.</t>
+          <t>I'm interested in hypersonic flow and heat shields and quantum sensing.</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Chess / board games;Running;Volunteering;</t>
+          <t>Lifting;Running;</t>
         </is>
       </c>
       <c r="O22" t="inlineStr"/>
@@ -2089,57 +2089,57 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>35</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>["Grad school planning", "Choosing a major", "Academics &amp; study habits"]</t>
+          <t>["Grad school planning", "Leadership &amp; military training", "AF/SF career planning"]</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>["Chemistry"]</t>
+          <t>["History"]</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>["Global Logistics", "Foreign language", "Space Studies"]</t>
+          <t>["Philosophy"]</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>["Master's right after graduation", "Rhodes"]</t>
+          <t>["Master's right after graduation", "Marshall", "Law school"]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>["Pilot", "Weather", "Developmental Engineer"]</t>
+          <t>["Medical", "Scientist", "RPA Pilot"]</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>["Entrepreneurship", "Career military"]</t>
+          <t>["Government / policy", "Not sure yet"]</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>["Internships", "Publishing research"]</t>
+          <t>["Competition teams / clubs"]</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>["Aerospace / hypersonics", "National security / policy", "Quantum / physics"]</t>
+          <t>["Ethics / philosophy", "Aerospace / hypersonics"]</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>I'm interested in hypersonic flow and heat shields and cyber defense of space systems.</t>
+          <t>I'm interested in cyber defense of space systems and renewable energy on bases.</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>["Climbing", "Reading"]</t>
+          <t>["Lifting", "Music"]</t>
         </is>
       </c>
       <c r="O23" t="inlineStr"/>
@@ -2162,57 +2162,57 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Grad school planning;Wellness &amp; balance;Leadership &amp; military training;</t>
+          <t>Fellowships &amp; scholarships;Research opportunities;AF/SF career planning;</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Systems Engineering;Foreign Area Studies;</t>
+          <t>Philosophy;Operations Research;Economics;</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>None / undecided;</t>
+          <t>Religion Studies;Foreign language;Space Studies;</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Schwarzman;Not sure yet;Rhodes;</t>
+          <t>Hertz / NSF GRFP;</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Undecided;Intelligence;RPA Pilot;</t>
+          <t>Air Battle Manager;Intelligence;</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Academia / research;Not sure yet;Law;</t>
+          <t>NGO / nonprofit;Entrepreneurship;Medicine;</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Soaring / powered flight;Study abroad / exchange semester;Summer research;</t>
+          <t>Soaring / powered flight;Competition teams / clubs;Publishing research;</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Autonomy / drones;Climate / environment;</t>
+          <t>Space;Biomedical / human performance;</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>I'm interested in Cold War nuclear strategy and renewable energy on bases.</t>
+          <t>I'm interested in Cold War nuclear strategy and hypersonic flow and heat shields.</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Music;</t>
+          <t>Running;Writing;</t>
         </is>
       </c>
       <c r="O24" t="inlineStr"/>
@@ -2235,17 +2235,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>["Time management", "AF/SF career planning"]</t>
+          <t>["Time management"]</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>["History", "Physics"]</t>
+          <t>["Data Science", "Foreign Area Studies"]</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2255,37 +2255,37 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>["Marshall", "Hertz / NSF GRFP"]</t>
+          <t>["PhD"]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>["Acquisitions / Program Management"]</t>
+          <t>["Space Operations"]</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>["Industry / tech", "Law"]</t>
+          <t>["Not sure yet", "Entrepreneurship", "Academia / research"]</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>["Competition teams / clubs", "Soaring / powered flight", "Cadet leadership positions"]</t>
+          <t>["Conferences / presenting"]</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>["Biomedical / human performance"]</t>
+          <t>["Not interested in research", "Quantum / physics", "Psychology / leadership"]</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>I'm interested in hypersonic flow and heat shields and leadership psychology under stress.</t>
+          <t>I'm interested in hypersonic flow and heat shields and human performance and sleep.</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>["Skiing / snowboarding"]</t>
+          <t>["Film / TV"]</t>
         </is>
       </c>
       <c r="O25" t="inlineStr"/>
@@ -2308,57 +2308,57 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>32</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Research opportunities;Fellowships &amp; scholarships;</t>
+          <t>Academics &amp; study habits;Fellowships &amp; scholarships;</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Space Operations;Meteorology;Legal Studies;</t>
+          <t>Humanities;</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Philosophy;Global Logistics;</t>
+          <t>None / undecided;Space Studies;Religion Studies;</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Truman;Hertz / NSF GRFP;</t>
+          <t>Fulbright;Mitchell;Gates Cambridge;</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Maintenance / Logistics;Pilot;</t>
+          <t>Special Warfare;Air Battle Manager;</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Career military;</t>
+          <t>Career military;Medicine;</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Competition teams / clubs;Cadet leadership positions;</t>
+          <t>Cadet leadership positions;Internships;</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Cybersecurity;Biomedical / human performance;</t>
+          <t>AI / machine learning;</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>I'm interested in human performance and sleep and quantum sensing.</t>
+          <t>I'm interested in Cold War nuclear strategy and Cold War nuclear strategy.</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Hiking / outdoors;Art / photography;</t>
+          <t>Climbing;Faith community;</t>
         </is>
       </c>
       <c r="O26" t="inlineStr"/>
@@ -2381,57 +2381,57 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>["Research opportunities", "Navigating cadet life"]</t>
+          <t>["Choosing a major", "Research opportunities", "Navigating cadet life"]</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>["Computer Science"]</t>
+          <t>["Systems Engineering", "Astronautical Engineering"]</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>["Foreign language", "Global Logistics", "Religion Studies"]</t>
+          <t>["Philosophy", "Foreign language"]</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>["Gates Cambridge", "Marshall"]</t>
+          <t>["Schwarzman", "Medical school", "Fulbright"]</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>["Maintenance / Logistics", "Finance / Contracting"]</t>
+          <t>["Scientist"]</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>["Medicine"]</t>
+          <t>["Not sure yet", "Medicine"]</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>["Soaring / powered flight", "Summer research"]</t>
+          <t>["Jump"]</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>["Space", "AI / machine learning"]</t>
+          <t>["AI / machine learning", "Ethics / philosophy"]</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>I'm interested in renewable energy on bases and Cold War nuclear strategy.</t>
+          <t>I'm interested in great power competition and great power competition.</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>["Skiing / snowboarding", "Gaming", "Chess / board games"]</t>
+          <t>["Climbing"]</t>
         </is>
       </c>
       <c r="O27" t="inlineStr"/>
@@ -2454,57 +2454,57 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Research opportunities;Grad school planning;Wellness &amp; balance;</t>
+          <t>Navigating cadet life;Leadership &amp; military training;Fellowships &amp; scholarships;</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Undecided;Aeronautical Engineering;</t>
+          <t>Systems Engineering;Economics;Humanities;</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Other;Nuclear Weapons &amp; Strategy;None / undecided;</t>
+          <t>Religion Studies;</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Law school;</t>
+          <t>Hertz / NSF GRFP;</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Combat Systems Officer;</t>
+          <t>Special Warfare;Acquisitions / Program Management;</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Law;Government / policy;Entrepreneurship;</t>
+          <t>Entrepreneurship;Not sure yet;</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Soaring / powered flight;</t>
+          <t>Ops Air Force;Soaring / powered flight;</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Autonomy / drones;Psychology / leadership;</t>
+          <t>Ethics / philosophy;Space;</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>I'm interested in great power competition and machine learning for satellite imagery.</t>
+          <t>I'm interested in machine learning for satellite imagery and renewable energy on bases.</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Film / TV;</t>
+          <t>Climbing;</t>
         </is>
       </c>
       <c r="O28" t="inlineStr"/>
@@ -2527,57 +2527,57 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>["AF/SF career planning", "Wellness &amp; balance"]</t>
+          <t>["Leadership &amp; military training", "Time management", "Grad school planning"]</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>["Philosophy", "Meteorology"]</t>
+          <t>["Electrical &amp; Computer Engineering", "Physics"]</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>["Other", "Global Logistics"]</t>
+          <t>["Other", "Philosophy"]</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>["Schwarzman"]</t>
+          <t>["Truman", "Not planning grad school", "Marshall"]</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>["Weather", "Maintenance / Logistics"]</t>
+          <t>["Special Warfare"]</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>["Academia / research"]</t>
+          <t>["Industry / tech", "Medicine", "Not sure yet"]</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>["Study abroad / exchange semester", "Internships", "Ops Air Force"]</t>
+          <t>["Soaring / powered flight", "Ops Air Force"]</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>["Education", "Quantum / physics", "Space"]</t>
+          <t>["Economics"]</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>I'm interested in cyber defense of space systems and human performance and sleep.</t>
+          <t>I'm interested in quantum sensing and quantum sensing.</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>["Volunteering", "Skiing / snowboarding"]</t>
+          <t>["Chess / board games", "Music", "Film / TV"]</t>
         </is>
       </c>
       <c r="O29" t="inlineStr"/>

</xml_diff>